<commit_message>
docs: list the nine college Department Head accounts on the staging site in the QA sheet and the member guide
Co-Authored-By: John Carlo Borgueta <johncarloborgueta@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/QA_TEST_SHEET.xlsx
+++ b/docs/QA_TEST_SHEET.xlsx
@@ -79,10 +79,10 @@
     <t>Department Head</t>
   </si>
   <si>
-    <t>940001 to 940005</t>
-  </si>
-  <si>
-    <t>940001 College of Computer Studies, 940002 Business, 940003 Teacher Education, 940004 Health Sciences, 940005 Engineering. One head per college.</t>
+    <t>940001 to 940009</t>
+  </si>
+  <si>
+    <t>940001 College of Computer Studies, 940002 Business Education, 940003 Teacher Education, 940004 Health Sciences, 940005 Engineering, 940006 Criminal Justice Education, 940007 Hospitality, Tourism and Customs Administration, 940008 Maritime Education, 940009 Nursing. One head per college; pick the college you were assigned.</t>
   </si>
   <si>
     <t>Admin (Organization Admin)</t>
@@ -16800,7 +16800,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{CE5A777F-A384-4E98-9685-6256870C8AA0}</x14:id>
+          <x14:id>{18821852-7557-4B39-ABAF-B05BB435070A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -16811,7 +16811,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{CE5A777F-A384-4E98-9685-6256870C8AA0}">
+          <x14:cfRule type="dataBar" id="{18821852-7557-4B39-ABAF-B05BB435070A}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>